<commit_message>
Populate workbook with Phase 4 market data
</commit_message>
<xml_diff>
--- a/models/builds/2026-08-07-Ritschard-pharma-exporter-model.xlsx
+++ b/models/builds/2026-08-07-Ritschard-pharma-exporter-model.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R7d306da47e8b4d5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend-Key" sheetId="2" r:id="R2a26d131c3844879"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="3" r:id="Rc00351cfcf0e464a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forward-Hedge" sheetId="4" r:id="R0fe221d893d2435e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Money-Market-Hedge" sheetId="5" r:id="R59da9a00dc56495e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options-Hedge" sheetId="6" r:id="R86afa386fad04827"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="R496c8d8b18a749f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes-Assumptions" sheetId="8" r:id="Rbb5bfb6310d0470a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="Rf22dbe3b10fe4c31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend-Key" sheetId="2" r:id="Re83c82e6764c4c83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="3" r:id="Ra159a9cc96db4253"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forward-Hedge" sheetId="4" r:id="R84a96c2fb9a149dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Money-Market-Hedge" sheetId="5" r:id="Rf7a17c825b9d4a1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options-Hedge" sheetId="6" r:id="R6fe46327e2424236"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="Radbc82e80f014320"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes-Assumptions" sheetId="8" r:id="R983f2b59ec6a4d79"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="FC_AMT">Inputs!$B$4</x:definedName>
@@ -360,6 +360,7 @@
     <c:plotArea>
       <c:lineChart>
         <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
@@ -591,7 +592,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf4282172d7f244ce"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbd8df12f563240d5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1069,7 +1070,7 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="62" t="str">
-        <x:v>Phase 2/3 market values are indicative modeling placeholders unless identified as scenario-provided. Phase 4 will replace the appropriate market inputs with live data and documented sources. FC_AMT and the indicative forward are scenario-provided; option premiums remain scenario assumptions in Phase 4.</x:v>
+        <x:v>Phase 4 populated workbook. Market inputs S0_in, R_USD, R_FC, F0_in, K_PUT, and K_CALL have been updated from the documented Phase 4 market-data process. FC_AMT and T_DAYS remain scenario inputs; PREM_PUT and PREM_CALL remain modeling assumptions as directed.</x:v>
       </x:c>
       <x:c r="B13" s="62"/>
       <x:c r="C13" s="62"/>
@@ -2141,7 +2142,7 @@
         <x:v>Foreign-currency receivable</x:v>
       </x:c>
       <x:c r="E4" s="60" t="str">
-        <x:v>Assigned scenario; remains fixed</x:v>
+        <x:v>Assigned FIN 321 Scenario #2; unchanged</x:v>
       </x:c>
       <x:c r="F4" s="60"/>
       <x:c r="G4" s="60"/>
@@ -2161,7 +2162,7 @@
         <x:v>S0_in</x:v>
       </x:c>
       <x:c r="B5" s="75" t="n">
-        <x:v>1.09</x:v>
+        <x:v>1.1535</x:v>
       </x:c>
       <x:c r="C5" s="60" t="str">
         <x:v>USD/EUR</x:v>
@@ -2170,7 +2171,7 @@
         <x:v>Current spot exchange rate</x:v>
       </x:c>
       <x:c r="E5" s="60" t="str">
-        <x:v>Indicative placeholder; replace with live EURUSD spot</x:v>
+        <x:v>ECB EUR/USD reference rate, August 7, 2026</x:v>
       </x:c>
       <x:c r="F5" s="60"/>
       <x:c r="G5" s="60"/>
@@ -2190,7 +2191,7 @@
         <x:v>F0_in</x:v>
       </x:c>
       <x:c r="B6" s="75" t="n">
-        <x:v>1.089</x:v>
+        <x:v>1.1747</x:v>
       </x:c>
       <x:c r="C6" s="60" t="str">
         <x:v>USD/EUR</x:v>
@@ -2199,7 +2200,7 @@
         <x:v>1-year forward rate</x:v>
       </x:c>
       <x:c r="E6" s="60" t="str">
-        <x:v>Scenario-provided indicative; replace with live quote or CIP-implied forward</x:v>
+        <x:v>CIP-implied from Phase 4 S0_in, R_USD, R_FC, and T_DAYS</x:v>
       </x:c>
       <x:c r="F6" s="60"/>
       <x:c r="G6" s="60"/>
@@ -2219,7 +2220,7 @@
         <x:v>R_USD</x:v>
       </x:c>
       <x:c r="B7" s="75" t="n">
-        <x:v>0.029</x:v>
+        <x:v>0.0406</x:v>
       </x:c>
       <x:c r="C7" s="60" t="str">
         <x:v>decimal annual</x:v>
@@ -2228,7 +2229,7 @@
         <x:v>1-year USD interest rate</x:v>
       </x:c>
       <x:c r="E7" s="60" t="str">
-        <x:v>Indicative placeholder; replace with live USD rate</x:v>
+        <x:v>1-Year U.S. Treasury Constant Maturity Rate; latest observation used</x:v>
       </x:c>
       <x:c r="F7" s="60"/>
       <x:c r="G7" s="60"/>
@@ -2248,7 +2249,7 @@
         <x:v>R_FC</x:v>
       </x:c>
       <x:c r="B8" s="75" t="n">
-        <x:v>0.03</x:v>
+        <x:v>0.02185</x:v>
       </x:c>
       <x:c r="C8" s="60" t="str">
         <x:v>decimal annual</x:v>
@@ -2257,7 +2258,7 @@
         <x:v>1-year EUR interest rate</x:v>
       </x:c>
       <x:c r="E8" s="60" t="str">
-        <x:v>Indicative placeholder; replace with live EUR rate</x:v>
+        <x:v>ECB €STR reference-rate proxy; latest published observation used</x:v>
       </x:c>
       <x:c r="F8" s="60"/>
       <x:c r="G8" s="60"/>
@@ -2277,7 +2278,7 @@
         <x:v>K_PUT</x:v>
       </x:c>
       <x:c r="B9" s="75" t="n">
-        <x:v>1.09</x:v>
+        <x:v>1.1535</x:v>
       </x:c>
       <x:c r="C9" s="60" t="str">
         <x:v>USD/EUR</x:v>
@@ -2286,7 +2287,7 @@
         <x:v>EUR put strike</x:v>
       </x:c>
       <x:c r="E9" s="60" t="str">
-        <x:v>Indicative placeholder; set at/near live spot</x:v>
+        <x:v>Set at live spot (ATM)</x:v>
       </x:c>
       <x:c r="F9" s="60"/>
       <x:c r="G9" s="60"/>
@@ -2306,7 +2307,7 @@
         <x:v>K_CALL</x:v>
       </x:c>
       <x:c r="B10" s="75" t="n">
-        <x:v>1.09</x:v>
+        <x:v>1.1535</x:v>
       </x:c>
       <x:c r="C10" s="60" t="str">
         <x:v>USD/EUR</x:v>
@@ -2315,7 +2316,7 @@
         <x:v>EUR call strike</x:v>
       </x:c>
       <x:c r="E10" s="60" t="str">
-        <x:v>Indicative placeholder; set at/near live spot</x:v>
+        <x:v>Set at live spot (ATM)</x:v>
       </x:c>
       <x:c r="F10" s="60"/>
       <x:c r="G10" s="60"/>
@@ -2344,7 +2345,7 @@
         <x:v>Put premium</x:v>
       </x:c>
       <x:c r="E11" s="60" t="str">
-        <x:v>Scenario assumption; retain at Phase 4</x:v>
+        <x:v>Phase 3 modeling assumption retained per Phase 4 instructions</x:v>
       </x:c>
       <x:c r="F11" s="60"/>
       <x:c r="G11" s="60"/>
@@ -2373,7 +2374,7 @@
         <x:v>Call premium</x:v>
       </x:c>
       <x:c r="E12" s="60" t="str">
-        <x:v>Scenario assumption; retain at Phase 4</x:v>
+        <x:v>Phase 3 modeling assumption retained per Phase 4 instructions</x:v>
       </x:c>
       <x:c r="F12" s="60"/>
       <x:c r="G12" s="60"/>
@@ -2402,7 +2403,7 @@
         <x:v>Time to maturity</x:v>
       </x:c>
       <x:c r="E13" s="60" t="str">
-        <x:v>Assigned one-year scenario</x:v>
+        <x:v>Assigned one-year scenario / ACT-360 convention</x:v>
       </x:c>
       <x:c r="F13" s="60"/>
       <x:c r="G13" s="60"/>
@@ -2849,7 +2850,7 @@
       </x:c>
       <x:c r="B5" s="81" t="n">
         <x:f>F0_in</x:f>
-        <x:v>1.089</x:v>
+        <x:v>1.1747</x:v>
       </x:c>
       <x:c r="C5" s="60"/>
       <x:c r="D5" s="60"/>
@@ -2873,7 +2874,7 @@
       </x:c>
       <x:c r="B6" s="82" t="n">
         <x:f>FC_AMT*F0_in</x:f>
-        <x:v>8712000</x:v>
+        <x:v>9397600</x:v>
       </x:c>
       <x:c r="C6" s="60"/>
       <x:c r="D6" s="60"/>
@@ -3432,7 +3433,7 @@
       </x:c>
       <x:c r="B4" s="80" t="n">
         <x:f>FC_AMT/(1+R_FC*T_DAYS/360)</x:f>
-        <x:v>7766990.291262136</x:v>
+        <x:v>7828937.711014337</x:v>
       </x:c>
       <x:c r="C4" s="60"/>
       <x:c r="D4" s="60"/>
@@ -3456,7 +3457,7 @@
       </x:c>
       <x:c r="B5" s="86" t="n">
         <x:f>B4*S0_in</x:f>
-        <x:v>8466019.417475728</x:v>
+        <x:v>9030679.649655037</x:v>
       </x:c>
       <x:c r="C5" s="60"/>
       <x:c r="D5" s="60"/>
@@ -3480,7 +3481,7 @@
       </x:c>
       <x:c r="B6" s="86" t="n">
         <x:f>B5*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>8711533.980582524</x:v>
+        <x:v>9397325.243431032</x:v>
       </x:c>
       <x:c r="C6" s="60"/>
       <x:c r="D6" s="60"/>
@@ -3523,7 +3524,7 @@
       </x:c>
       <x:c r="B8" s="81" t="n">
         <x:f>S0_in*(1+R_USD*T_DAYS/360)/(1+R_FC*T_DAYS/360)</x:f>
-        <x:v>1.0889417475728156</x:v>
+        <x:v>1.174665655428879</x:v>
       </x:c>
       <x:c r="C8" s="60"/>
       <x:c r="D8" s="60"/>
@@ -3547,7 +3548,7 @@
       </x:c>
       <x:c r="B9" s="81" t="n">
         <x:f>F0_in-B8</x:f>
-        <x:v>0.00005825242718437984</x:v>
+        <x:v>0.00003434457112105882</x:v>
       </x:c>
       <x:c r="C9" s="60"/>
       <x:c r="D9" s="60"/>
@@ -3571,7 +3572,7 @@
       </x:c>
       <x:c r="B10" s="87" t="n">
         <x:f>ABS(F0_in-B8)/F0_in</x:f>
-        <x:v>0.000053491668672525106</x:v>
+        <x:v>0.000029236886967786513</x:v>
       </x:c>
       <x:c r="C10" s="60"/>
       <x:c r="D10" s="60"/>
@@ -4063,7 +4064,7 @@
       </x:c>
       <x:c r="B4" s="81" t="n">
         <x:f>S0_in</x:f>
-        <x:v>1.09</x:v>
+        <x:v>1.1535</x:v>
       </x:c>
       <x:c r="C4" s="60"/>
       <x:c r="D4" s="60"/>
@@ -4106,7 +4107,7 @@
       </x:c>
       <x:c r="B6" s="81" t="n">
         <x:f>MAX(K_PUT,B4)</x:f>
-        <x:v>1.09</x:v>
+        <x:v>1.1535</x:v>
       </x:c>
       <x:c r="C6" s="60"/>
       <x:c r="D6" s="60"/>
@@ -4130,7 +4131,7 @@
       </x:c>
       <x:c r="B7" s="86" t="n">
         <x:f>FC_AMT*MAX(K_PUT,B4)</x:f>
-        <x:v>8720000</x:v>
+        <x:v>9228000</x:v>
       </x:c>
       <x:c r="C7" s="60"/>
       <x:c r="D7" s="60"/>
@@ -4177,8 +4178,8 @@
         <x:v>Put Premium at Maturity</x:v>
       </x:c>
       <x:c r="B9" s="86" t="n">
-        <x:f>FC_AMT*PREM_PUT*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>164640</x:v>
+        <x:f>FC_AMT*PREM_PUT</x:f>
+        <x:v>160000</x:v>
       </x:c>
       <x:c r="C9" s="60"/>
       <x:c r="D9" s="60"/>
@@ -4201,8 +4202,8 @@
         <x:v>Put Net USD Proceeds</x:v>
       </x:c>
       <x:c r="B10" s="82" t="n">
-        <x:f>FC_AMT*MAX(K_PUT,B4)-B9</x:f>
-        <x:v>8555360</x:v>
+        <x:f>FC_AMT*MAX(K_PUT,B4)-B8</x:f>
+        <x:v>9068000</x:v>
       </x:c>
       <x:c r="C10" s="60"/>
       <x:c r="D10" s="60"/>
@@ -4269,7 +4270,7 @@
       </x:c>
       <x:c r="B13" s="86" t="n">
         <x:f>FC_AMT*B4+FC_AMT*MAX(B4-K_CALL,0)</x:f>
-        <x:v>8720000</x:v>
+        <x:v>9228000</x:v>
       </x:c>
       <x:c r="C13" s="60"/>
       <x:c r="D13" s="60"/>
@@ -4316,8 +4317,8 @@
         <x:v>Call Premium at Maturity</x:v>
       </x:c>
       <x:c r="B15" s="86" t="n">
-        <x:f>FC_AMT*PREM_CALL*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>164640</x:v>
+        <x:f>FC_AMT*PREM_CALL</x:f>
+        <x:v>160000</x:v>
       </x:c>
       <x:c r="C15" s="60"/>
       <x:c r="D15" s="60"/>
@@ -4359,8 +4360,8 @@
         <x:v>Call Net USD Proceeds</x:v>
       </x:c>
       <x:c r="B17" s="82" t="n">
-        <x:f>FC_AMT*B4+FC_AMT*MAX(B4-K_CALL,0)-B15</x:f>
-        <x:v>8555360</x:v>
+        <x:f>FC_AMT*B4+FC_AMT*MAX(B4-K_CALL,0)-B14</x:f>
+        <x:v>9068000</x:v>
       </x:c>
       <x:c r="C17" s="60"/>
       <x:c r="D17" s="60"/>
@@ -4725,27 +4726,27 @@
       </x:c>
       <x:c r="B4" s="81" t="n">
         <x:f>S0_in*(1+A4)</x:f>
-        <x:v>1.0355</x:v>
+        <x:v>1.0958249999999998</x:v>
       </x:c>
       <x:c r="C4" s="86" t="n">
         <x:f>FC_AMT*B4</x:f>
-        <x:v>8284000.000000001</x:v>
+        <x:v>8766599.999999998</x:v>
       </x:c>
       <x:c r="D4" s="86" t="n">
         <x:f>FC_AMT*F0_in</x:f>
-        <x:v>8712000</x:v>
+        <x:v>9397600</x:v>
       </x:c>
       <x:c r="E4" s="86" t="n">
         <x:f>FC_AMT/(1+R_FC*T_DAYS/360)*S0_in*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>8711533.980582524</x:v>
+        <x:v>9397325.243431032</x:v>
       </x:c>
       <x:c r="F4" s="86" t="n">
-        <x:f>FC_AMT*MAX(K_PUT,B4)-FC_AMT*PREM_PUT*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>8555360</x:v>
+        <x:f>FC_AMT*MAX(K_PUT,B4)-FC_AMT*PREM_PUT</x:f>
+        <x:v>9068000</x:v>
       </x:c>
       <x:c r="G4" s="86" t="n">
-        <x:f>FC_AMT*B4+FC_AMT*MAX(B4-K_CALL,0)-FC_AMT*PREM_CALL*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>8119360.000000001</x:v>
+        <x:f>FC_AMT*B4+FC_AMT*MAX(B4-K_CALL,0)-FC_AMT*PREM_CALL</x:f>
+        <x:v>8606599.999999998</x:v>
       </x:c>
       <x:c r="H4" s="60"/>
       <x:c r="I4" s="60"/>
@@ -4764,27 +4765,27 @@
       </x:c>
       <x:c r="B5" s="81" t="n">
         <x:f>S0_in*(1+A5)</x:f>
-        <x:v>1.0464</x:v>
+        <x:v>1.10736</x:v>
       </x:c>
       <x:c r="C5" s="86" t="n">
         <x:f>FC_AMT*B5</x:f>
-        <x:v>8371200</x:v>
+        <x:v>8858880</x:v>
       </x:c>
       <x:c r="D5" s="86" t="n">
         <x:f>FC_AMT*F0_in</x:f>
-        <x:v>8712000</x:v>
+        <x:v>9397600</x:v>
       </x:c>
       <x:c r="E5" s="86" t="n">
         <x:f>FC_AMT/(1+R_FC*T_DAYS/360)*S0_in*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>8711533.980582524</x:v>
+        <x:v>9397325.243431032</x:v>
       </x:c>
       <x:c r="F5" s="86" t="n">
-        <x:f>FC_AMT*MAX(K_PUT,B5)-FC_AMT*PREM_PUT*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>8555360</x:v>
+        <x:f>FC_AMT*MAX(K_PUT,B5)-FC_AMT*PREM_PUT</x:f>
+        <x:v>9068000</x:v>
       </x:c>
       <x:c r="G5" s="86" t="n">
-        <x:f>FC_AMT*B5+FC_AMT*MAX(B5-K_CALL,0)-FC_AMT*PREM_CALL*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>8206560</x:v>
+        <x:f>FC_AMT*B5+FC_AMT*MAX(B5-K_CALL,0)-FC_AMT*PREM_CALL</x:f>
+        <x:v>8698880</x:v>
       </x:c>
       <x:c r="H5" s="60"/>
       <x:c r="I5" s="60"/>
@@ -4803,27 +4804,27 @@
       </x:c>
       <x:c r="B6" s="81" t="n">
         <x:f>S0_in*(1+A6)</x:f>
-        <x:v>1.0573000000000001</x:v>
+        <x:v>1.118895</x:v>
       </x:c>
       <x:c r="C6" s="86" t="n">
         <x:f>FC_AMT*B6</x:f>
-        <x:v>8458400.000000002</x:v>
+        <x:v>8951160</x:v>
       </x:c>
       <x:c r="D6" s="86" t="n">
         <x:f>FC_AMT*F0_in</x:f>
-        <x:v>8712000</x:v>
+        <x:v>9397600</x:v>
       </x:c>
       <x:c r="E6" s="86" t="n">
         <x:f>FC_AMT/(1+R_FC*T_DAYS/360)*S0_in*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>8711533.980582524</x:v>
+        <x:v>9397325.243431032</x:v>
       </x:c>
       <x:c r="F6" s="86" t="n">
-        <x:f>FC_AMT*MAX(K_PUT,B6)-FC_AMT*PREM_PUT*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>8555360</x:v>
+        <x:f>FC_AMT*MAX(K_PUT,B6)-FC_AMT*PREM_PUT</x:f>
+        <x:v>9068000</x:v>
       </x:c>
       <x:c r="G6" s="86" t="n">
-        <x:f>FC_AMT*B6+FC_AMT*MAX(B6-K_CALL,0)-FC_AMT*PREM_CALL*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>8293760.000000002</x:v>
+        <x:f>FC_AMT*B6+FC_AMT*MAX(B6-K_CALL,0)-FC_AMT*PREM_CALL</x:f>
+        <x:v>8791160</x:v>
       </x:c>
       <x:c r="H6" s="60"/>
       <x:c r="I6" s="60"/>
@@ -4842,27 +4843,27 @@
       </x:c>
       <x:c r="B7" s="81" t="n">
         <x:f>S0_in*(1+A7)</x:f>
-        <x:v>1.0682</x:v>
+        <x:v>1.13043</x:v>
       </x:c>
       <x:c r="C7" s="86" t="n">
         <x:f>FC_AMT*B7</x:f>
-        <x:v>8545600</x:v>
+        <x:v>9043440</x:v>
       </x:c>
       <x:c r="D7" s="86" t="n">
         <x:f>FC_AMT*F0_in</x:f>
-        <x:v>8712000</x:v>
+        <x:v>9397600</x:v>
       </x:c>
       <x:c r="E7" s="86" t="n">
         <x:f>FC_AMT/(1+R_FC*T_DAYS/360)*S0_in*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>8711533.980582524</x:v>
+        <x:v>9397325.243431032</x:v>
       </x:c>
       <x:c r="F7" s="86" t="n">
-        <x:f>FC_AMT*MAX(K_PUT,B7)-FC_AMT*PREM_PUT*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>8555360</x:v>
+        <x:f>FC_AMT*MAX(K_PUT,B7)-FC_AMT*PREM_PUT</x:f>
+        <x:v>9068000</x:v>
       </x:c>
       <x:c r="G7" s="86" t="n">
-        <x:f>FC_AMT*B7+FC_AMT*MAX(B7-K_CALL,0)-FC_AMT*PREM_CALL*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>8380960</x:v>
+        <x:f>FC_AMT*B7+FC_AMT*MAX(B7-K_CALL,0)-FC_AMT*PREM_CALL</x:f>
+        <x:v>8883440</x:v>
       </x:c>
       <x:c r="H7" s="60"/>
       <x:c r="I7" s="60"/>
@@ -4881,27 +4882,27 @@
       </x:c>
       <x:c r="B8" s="81" t="n">
         <x:f>S0_in*(1+A8)</x:f>
-        <x:v>1.0791000000000002</x:v>
+        <x:v>1.141965</x:v>
       </x:c>
       <x:c r="C8" s="86" t="n">
         <x:f>FC_AMT*B8</x:f>
-        <x:v>8632800.000000002</x:v>
+        <x:v>9135720</x:v>
       </x:c>
       <x:c r="D8" s="86" t="n">
         <x:f>FC_AMT*F0_in</x:f>
-        <x:v>8712000</x:v>
+        <x:v>9397600</x:v>
       </x:c>
       <x:c r="E8" s="86" t="n">
         <x:f>FC_AMT/(1+R_FC*T_DAYS/360)*S0_in*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>8711533.980582524</x:v>
+        <x:v>9397325.243431032</x:v>
       </x:c>
       <x:c r="F8" s="86" t="n">
-        <x:f>FC_AMT*MAX(K_PUT,B8)-FC_AMT*PREM_PUT*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>8555360</x:v>
+        <x:f>FC_AMT*MAX(K_PUT,B8)-FC_AMT*PREM_PUT</x:f>
+        <x:v>9068000</x:v>
       </x:c>
       <x:c r="G8" s="86" t="n">
-        <x:f>FC_AMT*B8+FC_AMT*MAX(B8-K_CALL,0)-FC_AMT*PREM_CALL*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>8468160.000000002</x:v>
+        <x:f>FC_AMT*B8+FC_AMT*MAX(B8-K_CALL,0)-FC_AMT*PREM_CALL</x:f>
+        <x:v>8975720</x:v>
       </x:c>
       <x:c r="H8" s="60"/>
       <x:c r="I8" s="60"/>
@@ -4920,27 +4921,27 @@
       </x:c>
       <x:c r="B9" s="81" t="n">
         <x:f>S0_in*(1+A9)</x:f>
-        <x:v>1.09</x:v>
+        <x:v>1.1535</x:v>
       </x:c>
       <x:c r="C9" s="86" t="n">
         <x:f>FC_AMT*B9</x:f>
-        <x:v>8720000</x:v>
+        <x:v>9228000</x:v>
       </x:c>
       <x:c r="D9" s="86" t="n">
         <x:f>FC_AMT*F0_in</x:f>
-        <x:v>8712000</x:v>
+        <x:v>9397600</x:v>
       </x:c>
       <x:c r="E9" s="86" t="n">
         <x:f>FC_AMT/(1+R_FC*T_DAYS/360)*S0_in*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>8711533.980582524</x:v>
+        <x:v>9397325.243431032</x:v>
       </x:c>
       <x:c r="F9" s="86" t="n">
-        <x:f>FC_AMT*MAX(K_PUT,B9)-FC_AMT*PREM_PUT*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>8555360</x:v>
+        <x:f>FC_AMT*MAX(K_PUT,B9)-FC_AMT*PREM_PUT</x:f>
+        <x:v>9068000</x:v>
       </x:c>
       <x:c r="G9" s="86" t="n">
-        <x:f>FC_AMT*B9+FC_AMT*MAX(B9-K_CALL,0)-FC_AMT*PREM_CALL*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>8555360</x:v>
+        <x:f>FC_AMT*B9+FC_AMT*MAX(B9-K_CALL,0)-FC_AMT*PREM_CALL</x:f>
+        <x:v>9068000</x:v>
       </x:c>
       <x:c r="H9" s="60"/>
       <x:c r="I9" s="60"/>
@@ -4959,27 +4960,27 @@
       </x:c>
       <x:c r="B10" s="81" t="n">
         <x:f>S0_in*(1+A10)</x:f>
-        <x:v>1.1009</x:v>
+        <x:v>1.165035</x:v>
       </x:c>
       <x:c r="C10" s="86" t="n">
         <x:f>FC_AMT*B10</x:f>
-        <x:v>8807200</x:v>
+        <x:v>9320280</x:v>
       </x:c>
       <x:c r="D10" s="86" t="n">
         <x:f>FC_AMT*F0_in</x:f>
-        <x:v>8712000</x:v>
+        <x:v>9397600</x:v>
       </x:c>
       <x:c r="E10" s="86" t="n">
         <x:f>FC_AMT/(1+R_FC*T_DAYS/360)*S0_in*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>8711533.980582524</x:v>
+        <x:v>9397325.243431032</x:v>
       </x:c>
       <x:c r="F10" s="86" t="n">
-        <x:f>FC_AMT*MAX(K_PUT,B10)-FC_AMT*PREM_PUT*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>8642560</x:v>
+        <x:f>FC_AMT*MAX(K_PUT,B10)-FC_AMT*PREM_PUT</x:f>
+        <x:v>9160280</x:v>
       </x:c>
       <x:c r="G10" s="86" t="n">
-        <x:f>FC_AMT*B10+FC_AMT*MAX(B10-K_CALL,0)-FC_AMT*PREM_CALL*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>8729760</x:v>
+        <x:f>FC_AMT*B10+FC_AMT*MAX(B10-K_CALL,0)-FC_AMT*PREM_CALL</x:f>
+        <x:v>9252560</x:v>
       </x:c>
       <x:c r="H10" s="60"/>
       <x:c r="I10" s="60"/>
@@ -4998,27 +4999,27 @@
       </x:c>
       <x:c r="B11" s="81" t="n">
         <x:f>S0_in*(1+A11)</x:f>
-        <x:v>1.1118000000000001</x:v>
+        <x:v>1.17657</x:v>
       </x:c>
       <x:c r="C11" s="86" t="n">
         <x:f>FC_AMT*B11</x:f>
-        <x:v>8894400.000000002</x:v>
+        <x:v>9412560</x:v>
       </x:c>
       <x:c r="D11" s="86" t="n">
         <x:f>FC_AMT*F0_in</x:f>
-        <x:v>8712000</x:v>
+        <x:v>9397600</x:v>
       </x:c>
       <x:c r="E11" s="86" t="n">
         <x:f>FC_AMT/(1+R_FC*T_DAYS/360)*S0_in*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>8711533.980582524</x:v>
+        <x:v>9397325.243431032</x:v>
       </x:c>
       <x:c r="F11" s="86" t="n">
-        <x:f>FC_AMT*MAX(K_PUT,B11)-FC_AMT*PREM_PUT*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>8729760.000000002</x:v>
+        <x:f>FC_AMT*MAX(K_PUT,B11)-FC_AMT*PREM_PUT</x:f>
+        <x:v>9252560</x:v>
       </x:c>
       <x:c r="G11" s="86" t="n">
-        <x:f>FC_AMT*B11+FC_AMT*MAX(B11-K_CALL,0)-FC_AMT*PREM_CALL*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>8904160.000000002</x:v>
+        <x:f>FC_AMT*B11+FC_AMT*MAX(B11-K_CALL,0)-FC_AMT*PREM_CALL</x:f>
+        <x:v>9437120</x:v>
       </x:c>
       <x:c r="H11" s="60"/>
       <x:c r="I11" s="60"/>
@@ -5037,27 +5038,27 @@
       </x:c>
       <x:c r="B12" s="81" t="n">
         <x:f>S0_in*(1+A12)</x:f>
-        <x:v>1.1227</x:v>
+        <x:v>1.188105</x:v>
       </x:c>
       <x:c r="C12" s="86" t="n">
         <x:f>FC_AMT*B12</x:f>
-        <x:v>8981600</x:v>
+        <x:v>9504840</x:v>
       </x:c>
       <x:c r="D12" s="86" t="n">
         <x:f>FC_AMT*F0_in</x:f>
-        <x:v>8712000</x:v>
+        <x:v>9397600</x:v>
       </x:c>
       <x:c r="E12" s="86" t="n">
         <x:f>FC_AMT/(1+R_FC*T_DAYS/360)*S0_in*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>8711533.980582524</x:v>
+        <x:v>9397325.243431032</x:v>
       </x:c>
       <x:c r="F12" s="86" t="n">
-        <x:f>FC_AMT*MAX(K_PUT,B12)-FC_AMT*PREM_PUT*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>8816960</x:v>
+        <x:f>FC_AMT*MAX(K_PUT,B12)-FC_AMT*PREM_PUT</x:f>
+        <x:v>9344840</x:v>
       </x:c>
       <x:c r="G12" s="86" t="n">
-        <x:f>FC_AMT*B12+FC_AMT*MAX(B12-K_CALL,0)-FC_AMT*PREM_CALL*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>9078560</x:v>
+        <x:f>FC_AMT*B12+FC_AMT*MAX(B12-K_CALL,0)-FC_AMT*PREM_CALL</x:f>
+        <x:v>9621680</x:v>
       </x:c>
       <x:c r="H12" s="60"/>
       <x:c r="I12" s="60"/>
@@ -5076,27 +5077,27 @@
       </x:c>
       <x:c r="B13" s="81" t="n">
         <x:f>S0_in*(1+A13)</x:f>
-        <x:v>1.1336000000000002</x:v>
+        <x:v>1.19964</x:v>
       </x:c>
       <x:c r="C13" s="86" t="n">
         <x:f>FC_AMT*B13</x:f>
-        <x:v>9068800.000000002</x:v>
+        <x:v>9597120</x:v>
       </x:c>
       <x:c r="D13" s="86" t="n">
         <x:f>FC_AMT*F0_in</x:f>
-        <x:v>8712000</x:v>
+        <x:v>9397600</x:v>
       </x:c>
       <x:c r="E13" s="86" t="n">
         <x:f>FC_AMT/(1+R_FC*T_DAYS/360)*S0_in*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>8711533.980582524</x:v>
+        <x:v>9397325.243431032</x:v>
       </x:c>
       <x:c r="F13" s="86" t="n">
-        <x:f>FC_AMT*MAX(K_PUT,B13)-FC_AMT*PREM_PUT*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>8904160.000000002</x:v>
+        <x:f>FC_AMT*MAX(K_PUT,B13)-FC_AMT*PREM_PUT</x:f>
+        <x:v>9437120</x:v>
       </x:c>
       <x:c r="G13" s="86" t="n">
-        <x:f>FC_AMT*B13+FC_AMT*MAX(B13-K_CALL,0)-FC_AMT*PREM_CALL*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>9252960.000000002</x:v>
+        <x:f>FC_AMT*B13+FC_AMT*MAX(B13-K_CALL,0)-FC_AMT*PREM_CALL</x:f>
+        <x:v>9806240</x:v>
       </x:c>
       <x:c r="H13" s="60"/>
       <x:c r="I13" s="60"/>
@@ -5115,27 +5116,27 @@
       </x:c>
       <x:c r="B14" s="81" t="n">
         <x:f>S0_in*(1+A14)</x:f>
-        <x:v>1.1445</x:v>
+        <x:v>1.2111750000000001</x:v>
       </x:c>
       <x:c r="C14" s="86" t="n">
         <x:f>FC_AMT*B14</x:f>
-        <x:v>9156000</x:v>
+        <x:v>9689400</x:v>
       </x:c>
       <x:c r="D14" s="86" t="n">
         <x:f>FC_AMT*F0_in</x:f>
-        <x:v>8712000</x:v>
+        <x:v>9397600</x:v>
       </x:c>
       <x:c r="E14" s="86" t="n">
         <x:f>FC_AMT/(1+R_FC*T_DAYS/360)*S0_in*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>8711533.980582524</x:v>
+        <x:v>9397325.243431032</x:v>
       </x:c>
       <x:c r="F14" s="86" t="n">
-        <x:f>FC_AMT*MAX(K_PUT,B14)-FC_AMT*PREM_PUT*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>8991360</x:v>
+        <x:f>FC_AMT*MAX(K_PUT,B14)-FC_AMT*PREM_PUT</x:f>
+        <x:v>9529400</x:v>
       </x:c>
       <x:c r="G14" s="86" t="n">
-        <x:f>FC_AMT*B14+FC_AMT*MAX(B14-K_CALL,0)-FC_AMT*PREM_CALL*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>9427360</x:v>
+        <x:f>FC_AMT*B14+FC_AMT*MAX(B14-K_CALL,0)-FC_AMT*PREM_CALL</x:f>
+        <x:v>9990800.000000002</x:v>
       </x:c>
       <x:c r="H14" s="60"/>
       <x:c r="I14" s="60"/>
@@ -5457,7 +5458,7 @@
     <x:mergeCell ref="A1:G1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93fcbb69d0364df0"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70018f567b0d4d95"/>
 </x:worksheet>
 </file>
 
@@ -5699,7 +5700,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B11" s="67" t="str">
-        <x:v>Option premiums are USD per EUR and are carried to maturity at R_USD for comparison.</x:v>
+        <x:v>Option premiums are quoted in USD per EUR and deducted directly from hedge proceeds without financing/carry, matching the FIN 321 FX Hedging Lab.</x:v>
       </x:c>
       <x:c r="C11" s="60"/>
       <x:c r="D11" s="60"/>
@@ -5876,11 +5877,11 @@
       </x:c>
       <x:c r="B19" s="86" t="n">
         <x:f>FC_AMT*F0_in</x:f>
-        <x:v>8712000</x:v>
+        <x:v>9397600</x:v>
       </x:c>
       <x:c r="C19" s="68" t="str">
         <x:f>IF(ABS(B19-8712000)&lt;1,"PASS","REVIEW")</x:f>
-        <x:v>PASS</x:v>
+        <x:v>REVIEW</x:v>
       </x:c>
       <x:c r="D19" s="60"/>
       <x:c r="E19" s="60"/>
@@ -5903,7 +5904,7 @@
       </x:c>
       <x:c r="B20" s="87" t="n">
         <x:f>ABS(F0_in-(S0_in*(1+R_USD*T_DAYS/360)/(1+R_FC*T_DAYS/360)))/F0_in</x:f>
-        <x:v>0.000053491668672525106</x:v>
+        <x:v>0.000029236886967786513</x:v>
       </x:c>
       <x:c r="C20" s="68" t="str">
         <x:f>IF(B20&lt;=0.001,"PASS","REVIEW")</x:f>
@@ -5930,7 +5931,7 @@
       </x:c>
       <x:c r="B21" s="86" t="n">
         <x:f>ABS(FC_AMT*F0_in-(FC_AMT/(1+R_FC*T_DAYS/360)*S0_in*(1+R_USD*T_DAYS/360)))</x:f>
-        <x:v>466.019417475909</x:v>
+        <x:v>274.75656896829605</x:v>
       </x:c>
       <x:c r="C21" s="68" t="str">
         <x:f>IF(B21&lt;=1000,"PASS","REVIEW")</x:f>
@@ -6011,7 +6012,7 @@
       </x:c>
       <x:c r="B24" s="87" t="n">
         <x:f>MIN(Sensitivity!B4:B14)/S0_in</x:f>
-        <x:v>0.95</x:v>
+        <x:v>0.9499999999999998</x:v>
       </x:c>
       <x:c r="C24" s="68" t="str">
         <x:f>IF(ABS(B24-0.95)&lt;0.000001,"PASS","REVIEW")</x:f>

</xml_diff>